<commit_message>
chore: update 1.0.0 pages
</commit_message>
<xml_diff>
--- a/branches/1.0.0/CodeSystem-mii-cs-sdd-ausbildung.xlsx
+++ b/branches/1.0.0/CodeSystem-mii-cs-sdd-ausbildung.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>1.0.0</t>
+    <t>2027.0.0-ballot.rc1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,25 +60,25 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-28T09:25:00+00:00</t>
+    <t>2026-08-31T15:46:48+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
   </si>
   <si>
-    <t>Medizininformatik-Initiative</t>
+    <t>NUM-DIZ</t>
   </si>
   <si>
     <t>Contact</t>
   </si>
   <si>
-    <t>Medizininformatik-Initiative (https://www.medizininformatik-initiative.de)</t>
+    <t>NUM-DIZ (https://www.netzwerk-universitaetsmedizin.de)</t>
   </si>
   <si>
     <t>Jurisdiction</t>
   </si>
   <si>
-    <t/>
+    <t>Germany</t>
   </si>
   <si>
     <t>Description</t>

</xml_diff>